<commit_message>
feat: aktueller Zwischenstand vor edoobox Copy-Workflow-Integration
</commit_message>
<xml_diff>
--- a/app/public/Kurstransfer/Planungstabellen Excel/Kurstransfer-werner-sql-lo-office.xlsx
+++ b/app/public/Kurstransfer/Planungstabellen Excel/Kurstransfer-werner-sql-lo-office.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\temp\Kursplan-Projekt\app\public\Kurstransfer\Planungstabellen Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A94103B-BE6A-4892-94AE-BA22CAF8D789}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B632ADF-03B4-466A-89BD-5E1C87C2A6D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30612" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Terminplanung 2027" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1336" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1336" uniqueCount="87">
   <si>
     <t>Datum</t>
   </si>
@@ -295,6 +295,9 @@
   </si>
   <si>
     <t>Impress Aufbau: Präsentationen professionalisieren und Master-Logik verstehen</t>
+  </si>
+  <si>
+    <t>Impress Umsteiger: Unterschiede zu Microsoft PowerPoint</t>
   </si>
 </sst>
 </file>
@@ -8279,8 +8282,8 @@
       <c r="A11" t="s">
         <v>65</v>
       </c>
-      <c r="B11" s="24" t="s">
-        <v>85</v>
+      <c r="B11" s="18" t="s">
+        <v>86</v>
       </c>
       <c r="C11" t="s">
         <v>77</v>

</xml_diff>